<commit_message>
Daily attendance processing - 2026-03-25 17:48:37 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -6130,7 +6130,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
@@ -8965,7 +8965,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
@@ -10825,7 +10825,7 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr">
@@ -14858,7 +14858,7 @@
       </c>
       <c r="G299" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H299" s="2" t="inlineStr">

</xml_diff>